<commit_message>
Update preliminary analysis files
</commit_message>
<xml_diff>
--- a/00_Data/Full_experiment/Full_experiment_S1.xlsx
+++ b/00_Data/Full_experiment/Full_experiment_S1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="802" documentId="8_{7A9B329B-35ED-3242-9754-4D2EFB164FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A303167C-1C5B-45A3-B2BB-C70257684C72}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{D787752A-2EF4-4C1F-98F1-137D096492FA}"/>
+    <workbookView xWindow="3040" yWindow="3040" windowWidth="28800" windowHeight="15370" activeTab="2" xr2:uid="{D787752A-2EF4-4C1F-98F1-137D096492FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Littoralis_S1" sheetId="1" r:id="rId1"/>
@@ -672,7 +672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -686,7 +686,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,6 +701,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4056,10 +4059,10 @@
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17">
         <v>10</v>
       </c>
-      <c r="K17" s="11">
+      <c r="K17">
         <v>20</v>
       </c>
       <c r="L17">
@@ -4243,10 +4246,10 @@
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18">
         <v>10</v>
       </c>
-      <c r="K18" s="11">
+      <c r="K18">
         <v>17</v>
       </c>
       <c r="L18">
@@ -4430,10 +4433,10 @@
         <f t="shared" si="3"/>
         <v>19</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19">
         <v>10</v>
       </c>
-      <c r="K19" s="11">
+      <c r="K19">
         <v>15</v>
       </c>
       <c r="L19">
@@ -4617,10 +4620,10 @@
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20">
         <v>10</v>
       </c>
-      <c r="K20" s="11">
+      <c r="K20">
         <v>13</v>
       </c>
       <c r="L20">
@@ -4804,10 +4807,10 @@
         <f t="shared" si="3"/>
         <v>19</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21">
         <v>10</v>
       </c>
-      <c r="K21" s="11">
+      <c r="K21">
         <v>17</v>
       </c>
       <c r="L21">
@@ -4991,10 +4994,10 @@
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22">
         <v>13</v>
       </c>
-      <c r="K22" s="11">
+      <c r="K22">
         <v>15</v>
       </c>
       <c r="L22">
@@ -5178,10 +5181,10 @@
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="J23" s="11">
+      <c r="J23">
         <v>13</v>
       </c>
-      <c r="K23" s="11">
+      <c r="K23">
         <v>22</v>
       </c>
       <c r="L23">
@@ -5365,10 +5368,10 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J24" s="11">
-        <v>0</v>
-      </c>
-      <c r="K24" s="11">
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
@@ -5552,10 +5555,10 @@
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="J25" s="11">
+      <c r="J25">
         <v>10</v>
       </c>
-      <c r="K25" s="11">
+      <c r="K25">
         <v>17</v>
       </c>
       <c r="L25">
@@ -5739,10 +5742,10 @@
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="J26" s="11">
+      <c r="J26">
         <v>13</v>
       </c>
-      <c r="K26" s="11">
+      <c r="K26">
         <v>17</v>
       </c>
       <c r="L26">
@@ -5926,10 +5929,10 @@
         <f t="shared" si="3"/>
         <v>19</v>
       </c>
-      <c r="J27" s="11">
+      <c r="J27">
         <v>10</v>
       </c>
-      <c r="K27" s="11">
+      <c r="K27">
         <v>13</v>
       </c>
       <c r="L27">
@@ -6113,10 +6116,10 @@
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="J28" s="11">
+      <c r="J28">
         <v>13</v>
       </c>
-      <c r="K28" s="11">
+      <c r="K28">
         <v>13</v>
       </c>
       <c r="L28">
@@ -6300,10 +6303,10 @@
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J29">
         <v>8</v>
       </c>
-      <c r="K29" s="11">
+      <c r="K29">
         <v>13</v>
       </c>
       <c r="L29">
@@ -6487,10 +6490,10 @@
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30">
         <v>10</v>
       </c>
-      <c r="K30" s="11">
+      <c r="K30">
         <v>17</v>
       </c>
       <c r="L30">
@@ -6861,10 +6864,10 @@
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="J32" s="11">
+      <c r="J32">
         <v>13</v>
       </c>
-      <c r="K32" s="11">
+      <c r="K32">
         <v>17</v>
       </c>
       <c r="L32">
@@ -7048,10 +7051,10 @@
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J33">
         <v>13</v>
       </c>
-      <c r="K33" s="11">
+      <c r="K33">
         <v>27</v>
       </c>
       <c r="L33">
@@ -7235,10 +7238,10 @@
         <f t="shared" ref="I34:I56" si="4">SUM(L34:AW34)</f>
         <v>14</v>
       </c>
-      <c r="J34" s="11">
+      <c r="J34">
         <v>13</v>
       </c>
-      <c r="K34" s="11">
+      <c r="K34">
         <v>17</v>
       </c>
       <c r="L34">
@@ -7422,10 +7425,10 @@
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
-      <c r="J35" s="11">
+      <c r="J35">
         <v>13</v>
       </c>
-      <c r="K35" s="11">
+      <c r="K35">
         <v>20</v>
       </c>
       <c r="L35">
@@ -7609,10 +7612,10 @@
         <f t="shared" si="4"/>
         <v>17</v>
       </c>
-      <c r="J36" s="11">
+      <c r="J36">
         <v>13</v>
       </c>
-      <c r="K36" s="11">
+      <c r="K36">
         <v>20</v>
       </c>
       <c r="L36">
@@ -7796,10 +7799,10 @@
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="J37" s="11">
+      <c r="J37">
         <v>10</v>
       </c>
-      <c r="K37" s="11">
+      <c r="K37">
         <v>20</v>
       </c>
       <c r="L37">
@@ -7983,10 +7986,10 @@
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
-      <c r="J38" s="11">
+      <c r="J38">
         <v>10</v>
       </c>
-      <c r="K38" s="11">
+      <c r="K38">
         <v>13</v>
       </c>
       <c r="L38">
@@ -8170,10 +8173,10 @@
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
-      <c r="J39" s="11">
+      <c r="J39">
         <v>10</v>
       </c>
-      <c r="K39" s="11">
+      <c r="K39">
         <v>17</v>
       </c>
       <c r="L39">
@@ -8357,10 +8360,10 @@
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="J40" s="11">
+      <c r="J40">
         <v>15</v>
       </c>
-      <c r="K40" s="11">
+      <c r="K40">
         <v>24</v>
       </c>
       <c r="L40">
@@ -8544,10 +8547,10 @@
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
-      <c r="J41" s="11">
+      <c r="J41">
         <v>13</v>
       </c>
-      <c r="K41" s="11">
+      <c r="K41">
         <v>29</v>
       </c>
       <c r="L41">
@@ -8731,10 +8734,10 @@
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="J42" s="11">
+      <c r="J42">
         <v>13</v>
       </c>
-      <c r="K42" s="11">
+      <c r="K42">
         <v>20</v>
       </c>
       <c r="L42">
@@ -8918,10 +8921,10 @@
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="J43" s="11">
+      <c r="J43">
         <v>17</v>
       </c>
-      <c r="K43" s="11">
+      <c r="K43">
         <v>17</v>
       </c>
       <c r="L43">
@@ -9105,10 +9108,10 @@
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="J44" s="11">
+      <c r="J44">
         <v>10</v>
       </c>
-      <c r="K44" s="11">
+      <c r="K44">
         <v>20</v>
       </c>
       <c r="L44">
@@ -9292,10 +9295,10 @@
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="J45" s="11">
+      <c r="J45">
         <v>10</v>
       </c>
-      <c r="K45" s="11">
+      <c r="K45">
         <v>17</v>
       </c>
       <c r="L45">
@@ -9666,10 +9669,10 @@
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
-      <c r="J47" s="11">
+      <c r="J47">
         <v>10</v>
       </c>
-      <c r="K47" s="11">
+      <c r="K47">
         <v>17</v>
       </c>
       <c r="L47">
@@ -9853,10 +9856,10 @@
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
-      <c r="J48" s="11">
+      <c r="J48">
         <v>8</v>
       </c>
-      <c r="K48" s="11">
+      <c r="K48">
         <v>17</v>
       </c>
       <c r="L48">
@@ -10040,10 +10043,10 @@
         <f t="shared" si="4"/>
         <v>17</v>
       </c>
-      <c r="J49" s="11">
+      <c r="J49">
         <v>10</v>
       </c>
-      <c r="K49" s="11">
+      <c r="K49">
         <v>13</v>
       </c>
       <c r="L49">
@@ -10227,10 +10230,10 @@
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="J50" s="11">
+      <c r="J50">
         <v>8</v>
       </c>
-      <c r="K50" s="11">
+      <c r="K50">
         <v>15</v>
       </c>
       <c r="L50">
@@ -10414,10 +10417,10 @@
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
-      <c r="J51" s="11">
+      <c r="J51">
         <v>8</v>
       </c>
-      <c r="K51" s="11">
+      <c r="K51">
         <v>20</v>
       </c>
       <c r="L51">
@@ -10601,10 +10604,10 @@
         <f t="shared" si="4"/>
         <v>17</v>
       </c>
-      <c r="J52" s="11">
+      <c r="J52">
         <v>10</v>
       </c>
-      <c r="K52" s="11">
+      <c r="K52">
         <v>15</v>
       </c>
       <c r="L52">
@@ -10788,10 +10791,10 @@
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
-      <c r="J53" s="11">
+      <c r="J53">
         <v>10</v>
       </c>
-      <c r="K53" s="11">
+      <c r="K53">
         <v>13</v>
       </c>
       <c r="L53">
@@ -10975,10 +10978,10 @@
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="J54" s="11">
+      <c r="J54">
         <v>8</v>
       </c>
-      <c r="K54" s="11">
+      <c r="K54">
         <v>13</v>
       </c>
       <c r="L54">
@@ -11162,10 +11165,10 @@
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
-      <c r="J55" s="11">
+      <c r="J55">
         <v>8</v>
       </c>
-      <c r="K55" s="11">
+      <c r="K55">
         <v>10</v>
       </c>
       <c r="L55">
@@ -11349,10 +11352,10 @@
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
-      <c r="J56" s="11">
+      <c r="J56">
         <v>8</v>
       </c>
-      <c r="K56" s="11">
+      <c r="K56">
         <v>13</v>
       </c>
       <c r="L56">
@@ -11536,10 +11539,10 @@
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="J57" s="11">
+      <c r="J57">
         <v>8</v>
       </c>
-      <c r="K57" s="11">
+      <c r="K57">
         <v>13</v>
       </c>
       <c r="L57">
@@ -11726,7 +11729,7 @@
       <c r="J58">
         <v>10</v>
       </c>
-      <c r="K58" s="11">
+      <c r="K58">
         <v>13</v>
       </c>
       <c r="L58">
@@ -11913,7 +11916,7 @@
       <c r="J59">
         <v>8</v>
       </c>
-      <c r="K59" s="11">
+      <c r="K59">
         <v>13</v>
       </c>
       <c r="L59">
@@ -12100,7 +12103,7 @@
       <c r="J60">
         <v>8</v>
       </c>
-      <c r="K60" s="11">
+      <c r="K60">
         <v>13</v>
       </c>
       <c r="L60">
@@ -12471,10 +12474,10 @@
         <f t="shared" si="5"/>
         <v>18</v>
       </c>
-      <c r="J62" s="11">
+      <c r="J62">
         <v>13</v>
       </c>
-      <c r="K62" s="11">
+      <c r="K62">
         <v>13</v>
       </c>
       <c r="L62">
@@ -12658,10 +12661,10 @@
         <f t="shared" si="5"/>
         <v>15</v>
       </c>
-      <c r="J63" s="11">
+      <c r="J63">
         <v>10</v>
       </c>
-      <c r="K63" s="11">
+      <c r="K63">
         <v>13</v>
       </c>
       <c r="L63">
@@ -12845,10 +12848,10 @@
         <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="J64" s="11">
+      <c r="J64">
         <v>10</v>
       </c>
-      <c r="K64" s="11">
+      <c r="K64">
         <v>10</v>
       </c>
       <c r="L64">
@@ -13032,10 +13035,10 @@
         <f t="shared" si="5"/>
         <v>20</v>
       </c>
-      <c r="J65" s="11">
+      <c r="J65">
         <v>10</v>
       </c>
-      <c r="K65" s="11">
+      <c r="K65">
         <v>17</v>
       </c>
       <c r="L65">
@@ -13219,10 +13222,10 @@
         <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="J66" s="11">
+      <c r="J66">
         <v>10</v>
       </c>
-      <c r="K66" s="11">
+      <c r="K66">
         <v>17</v>
       </c>
       <c r="L66">
@@ -13406,10 +13409,10 @@
         <f t="shared" si="5"/>
         <v>17</v>
       </c>
-      <c r="J67" s="11">
+      <c r="J67">
         <v>10</v>
       </c>
-      <c r="K67" s="11">
+      <c r="K67">
         <v>20</v>
       </c>
       <c r="L67">
@@ -13593,10 +13596,10 @@
         <f t="shared" si="5"/>
         <v>17</v>
       </c>
-      <c r="J68" s="11">
+      <c r="J68">
         <v>8</v>
       </c>
-      <c r="K68" s="11">
+      <c r="K68">
         <v>10</v>
       </c>
       <c r="L68">
@@ -13780,10 +13783,10 @@
         <f t="shared" si="5"/>
         <v>17</v>
       </c>
-      <c r="J69" s="11">
+      <c r="J69">
         <v>13</v>
       </c>
-      <c r="K69" s="11">
+      <c r="K69">
         <v>15</v>
       </c>
       <c r="L69">
@@ -13967,10 +13970,10 @@
         <f t="shared" si="5"/>
         <v>20</v>
       </c>
-      <c r="J70" s="11">
+      <c r="J70">
         <v>8</v>
       </c>
-      <c r="K70" s="11">
+      <c r="K70">
         <v>10</v>
       </c>
       <c r="L70">
@@ -14154,10 +14157,10 @@
         <f t="shared" si="5"/>
         <v>11</v>
       </c>
-      <c r="J71" s="11">
+      <c r="J71">
         <v>10</v>
       </c>
-      <c r="K71" s="11">
+      <c r="K71">
         <v>29</v>
       </c>
       <c r="L71">
@@ -14341,10 +14344,10 @@
         <f t="shared" si="5"/>
         <v>13</v>
       </c>
-      <c r="J72" s="11">
+      <c r="J72">
         <v>8</v>
       </c>
-      <c r="K72" s="11">
+      <c r="K72">
         <v>13</v>
       </c>
       <c r="L72">
@@ -14528,10 +14531,10 @@
         <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="J73" s="11">
+      <c r="J73">
         <v>8</v>
       </c>
-      <c r="K73" s="11">
+      <c r="K73">
         <v>13</v>
       </c>
       <c r="L73">
@@ -14715,10 +14718,10 @@
         <f t="shared" si="5"/>
         <v>20</v>
       </c>
-      <c r="J74" s="11">
+      <c r="J74">
         <v>8</v>
       </c>
-      <c r="K74" s="11">
+      <c r="K74">
         <v>13</v>
       </c>
       <c r="L74">
@@ -14902,10 +14905,10 @@
         <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="J75" s="11">
+      <c r="J75">
         <v>8</v>
       </c>
-      <c r="K75" s="11">
+      <c r="K75">
         <v>13</v>
       </c>
       <c r="L75">
@@ -15276,10 +15279,10 @@
         <f t="shared" si="5"/>
         <v>17</v>
       </c>
-      <c r="J77" s="11">
+      <c r="J77">
         <v>13</v>
       </c>
-      <c r="K77" s="11">
+      <c r="K77">
         <v>25</v>
       </c>
       <c r="L77">
@@ -15463,10 +15466,10 @@
         <f t="shared" ref="I78" si="7">SUM(L78:AX78)</f>
         <v>18</v>
       </c>
-      <c r="J78" s="11">
+      <c r="J78">
         <v>10</v>
       </c>
-      <c r="K78" s="11">
+      <c r="K78">
         <v>39</v>
       </c>
       <c r="L78">
@@ -15650,10 +15653,10 @@
         <f t="shared" ref="I79:I91" si="8">SUM(L79:AW79)</f>
         <v>14</v>
       </c>
-      <c r="J79" s="11">
+      <c r="J79">
         <v>13</v>
       </c>
-      <c r="K79" s="11">
+      <c r="K79">
         <v>17</v>
       </c>
       <c r="L79">
@@ -15837,10 +15840,10 @@
         <f t="shared" si="8"/>
         <v>18</v>
       </c>
-      <c r="J80" s="11">
+      <c r="J80">
         <v>13</v>
       </c>
-      <c r="K80" s="11">
+      <c r="K80">
         <v>20</v>
       </c>
       <c r="L80">
@@ -16024,10 +16027,10 @@
         <f t="shared" si="8"/>
         <v>17</v>
       </c>
-      <c r="J81" s="11">
+      <c r="J81">
         <v>15</v>
       </c>
-      <c r="K81" s="11">
+      <c r="K81">
         <v>24</v>
       </c>
       <c r="L81">
@@ -16211,10 +16214,10 @@
         <f t="shared" si="8"/>
         <v>19</v>
       </c>
-      <c r="J82" s="11">
+      <c r="J82">
         <v>19</v>
       </c>
-      <c r="K82" s="11">
+      <c r="K82">
         <v>15</v>
       </c>
       <c r="L82">
@@ -16398,10 +16401,10 @@
         <f t="shared" si="8"/>
         <v>19</v>
       </c>
-      <c r="J83" s="11">
+      <c r="J83">
         <v>19</v>
       </c>
-      <c r="K83" s="11">
+      <c r="K83">
         <v>13</v>
       </c>
       <c r="L83">
@@ -16585,10 +16588,10 @@
         <f t="shared" si="8"/>
         <v>19</v>
       </c>
-      <c r="J84" s="11">
+      <c r="J84">
         <v>19</v>
       </c>
-      <c r="K84" s="11">
+      <c r="K84">
         <v>13</v>
       </c>
       <c r="L84">
@@ -16772,10 +16775,10 @@
         <f t="shared" si="8"/>
         <v>14</v>
       </c>
-      <c r="J85" s="11">
+      <c r="J85">
         <v>13</v>
       </c>
-      <c r="K85" s="11">
+      <c r="K85">
         <v>20</v>
       </c>
       <c r="L85">
@@ -16959,10 +16962,10 @@
         <f t="shared" si="8"/>
         <v>17</v>
       </c>
-      <c r="J86" s="11">
+      <c r="J86">
         <v>13</v>
       </c>
-      <c r="K86" s="11">
+      <c r="K86">
         <v>17</v>
       </c>
       <c r="L86">
@@ -17146,10 +17149,10 @@
         <f t="shared" si="8"/>
         <v>18</v>
       </c>
-      <c r="J87" s="11">
+      <c r="J87">
         <v>13</v>
       </c>
-      <c r="K87" s="11">
+      <c r="K87">
         <v>20</v>
       </c>
       <c r="L87">
@@ -17333,10 +17336,10 @@
         <f t="shared" si="8"/>
         <v>17</v>
       </c>
-      <c r="J88" s="11">
+      <c r="J88">
         <v>13</v>
       </c>
-      <c r="K88" s="11">
+      <c r="K88">
         <v>15</v>
       </c>
       <c r="L88">
@@ -17520,10 +17523,10 @@
         <f t="shared" si="8"/>
         <v>15</v>
       </c>
-      <c r="J89" s="11">
+      <c r="J89">
         <v>13</v>
       </c>
-      <c r="K89" s="11">
+      <c r="K89">
         <v>13</v>
       </c>
       <c r="L89">
@@ -17707,10 +17710,10 @@
         <f t="shared" si="8"/>
         <v>17</v>
       </c>
-      <c r="J90" s="11">
+      <c r="J90">
         <v>13</v>
       </c>
-      <c r="K90" s="11">
+      <c r="K90">
         <v>15</v>
       </c>
       <c r="L90">
@@ -17894,10 +17897,10 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J91" s="11">
-        <v>0</v>
-      </c>
-      <c r="K91" s="11">
+      <c r="J91">
+        <v>0</v>
+      </c>
+      <c r="K91">
         <v>0</v>
       </c>
       <c r="L91">
@@ -21106,10 +21109,10 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17">
         <v>8</v>
       </c>
-      <c r="K17" s="11">
+      <c r="K17">
         <v>13</v>
       </c>
       <c r="L17">
@@ -21294,10 +21297,10 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18">
         <v>8</v>
       </c>
-      <c r="K18" s="11">
+      <c r="K18">
         <v>10</v>
       </c>
       <c r="L18">
@@ -21482,10 +21485,10 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19">
         <v>8</v>
       </c>
-      <c r="K19" s="11">
+      <c r="K19">
         <v>20</v>
       </c>
       <c r="L19">
@@ -21670,10 +21673,10 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20">
         <v>8</v>
       </c>
-      <c r="K20" s="11">
+      <c r="K20">
         <v>13</v>
       </c>
       <c r="L20">
@@ -21858,10 +21861,10 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21">
         <v>8</v>
       </c>
-      <c r="K21" s="11">
+      <c r="K21">
         <v>8</v>
       </c>
       <c r="L21">
@@ -22046,10 +22049,10 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22">
         <v>6</v>
       </c>
-      <c r="K22" s="11">
+      <c r="K22">
         <v>10</v>
       </c>
       <c r="L22">
@@ -22234,10 +22237,10 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="J23" s="11">
+      <c r="J23">
         <v>6</v>
       </c>
-      <c r="K23" s="11">
+      <c r="K23">
         <v>10</v>
       </c>
       <c r="L23">
@@ -22422,10 +22425,10 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="J24" s="11">
+      <c r="J24">
         <v>6</v>
       </c>
-      <c r="K24" s="11">
+      <c r="K24">
         <v>8</v>
       </c>
       <c r="L24">
@@ -22610,10 +22613,10 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="J25" s="11">
+      <c r="J25">
         <v>6</v>
       </c>
-      <c r="K25" s="11">
+      <c r="K25">
         <v>13</v>
       </c>
       <c r="L25">
@@ -22798,10 +22801,10 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="J26" s="11">
+      <c r="J26">
         <v>8</v>
       </c>
-      <c r="K26" s="11">
+      <c r="K26">
         <v>10</v>
       </c>
       <c r="L26">
@@ -22986,10 +22989,10 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="J27" s="11">
+      <c r="J27">
         <v>6</v>
       </c>
-      <c r="K27" s="11">
+      <c r="K27">
         <v>13</v>
       </c>
       <c r="L27">
@@ -23174,10 +23177,10 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="J28" s="11">
+      <c r="J28">
         <v>6</v>
       </c>
-      <c r="K28" s="11">
+      <c r="K28">
         <v>13</v>
       </c>
       <c r="L28">
@@ -23362,10 +23365,10 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J29">
         <v>6</v>
       </c>
-      <c r="K29" s="11">
+      <c r="K29">
         <v>8</v>
       </c>
       <c r="L29">
@@ -23550,10 +23553,10 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30">
         <v>6</v>
       </c>
-      <c r="K30" s="11">
+      <c r="K30">
         <v>13</v>
       </c>
       <c r="L30">
@@ -23926,10 +23929,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="J32" s="11">
+      <c r="J32">
         <v>10</v>
       </c>
-      <c r="K32" s="11">
+      <c r="K32">
         <v>15</v>
       </c>
       <c r="L32">
@@ -24114,10 +24117,10 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J33">
         <v>10</v>
       </c>
-      <c r="K33" s="11">
+      <c r="K33">
         <v>13</v>
       </c>
       <c r="L33">
@@ -24302,10 +24305,10 @@
         <f t="shared" ref="I34:I65" si="2">SUM(L34:AO34)</f>
         <v>12</v>
       </c>
-      <c r="J34" s="11">
+      <c r="J34">
         <v>10</v>
       </c>
-      <c r="K34" s="11">
+      <c r="K34">
         <v>13</v>
       </c>
       <c r="L34">
@@ -24490,10 +24493,10 @@
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J35" s="11">
+      <c r="J35">
         <v>8</v>
       </c>
-      <c r="K35" s="11">
+      <c r="K35">
         <v>13</v>
       </c>
       <c r="L35">
@@ -24678,10 +24681,10 @@
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="J36" s="11">
+      <c r="J36">
         <v>8</v>
       </c>
-      <c r="K36" s="11">
+      <c r="K36">
         <v>10</v>
       </c>
       <c r="L36">
@@ -24866,10 +24869,10 @@
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="J37" s="11">
+      <c r="J37">
         <v>10</v>
       </c>
-      <c r="K37" s="11">
+      <c r="K37">
         <v>22</v>
       </c>
       <c r="L37">
@@ -25054,10 +25057,10 @@
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="J38" s="11">
+      <c r="J38">
         <v>10</v>
       </c>
-      <c r="K38" s="11">
+      <c r="K38">
         <v>13</v>
       </c>
       <c r="L38">
@@ -25242,10 +25245,10 @@
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="J39" s="11">
+      <c r="J39">
         <v>13</v>
       </c>
-      <c r="K39" s="11">
+      <c r="K39">
         <v>17</v>
       </c>
       <c r="L39">
@@ -25430,10 +25433,10 @@
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="J40" s="11">
+      <c r="J40">
         <v>8</v>
       </c>
-      <c r="K40" s="11">
+      <c r="K40">
         <v>12</v>
       </c>
       <c r="L40">
@@ -25618,10 +25621,10 @@
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="J41" s="11">
+      <c r="J41">
         <v>13</v>
       </c>
-      <c r="K41" s="11">
+      <c r="K41">
         <v>17</v>
       </c>
       <c r="L41">
@@ -25806,10 +25809,10 @@
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="J42" s="11">
+      <c r="J42">
         <v>13</v>
       </c>
-      <c r="K42" s="11">
+      <c r="K42">
         <v>17</v>
       </c>
       <c r="L42">
@@ -25994,10 +25997,10 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="J43" s="11">
+      <c r="J43">
         <v>13</v>
       </c>
-      <c r="K43" s="11">
+      <c r="K43">
         <v>13</v>
       </c>
       <c r="L43">
@@ -26182,10 +26185,10 @@
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J44" s="11">
+      <c r="J44">
         <v>8</v>
       </c>
-      <c r="K44" s="11">
+      <c r="K44">
         <v>13</v>
       </c>
       <c r="L44">
@@ -26370,10 +26373,10 @@
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="J45" s="11">
+      <c r="J45">
         <v>8</v>
       </c>
-      <c r="K45" s="11">
+      <c r="K45">
         <v>8</v>
       </c>
       <c r="L45">
@@ -26746,10 +26749,10 @@
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="J47" s="11">
+      <c r="J47">
         <v>8</v>
       </c>
-      <c r="K47" s="11">
+      <c r="K47">
         <v>13</v>
       </c>
       <c r="L47">
@@ -26934,10 +26937,10 @@
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J48" s="11">
+      <c r="J48">
         <v>8</v>
       </c>
-      <c r="K48" s="11">
+      <c r="K48">
         <v>13</v>
       </c>
       <c r="L48">
@@ -27122,10 +27125,10 @@
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J49" s="11">
+      <c r="J49">
         <v>8</v>
       </c>
-      <c r="K49" s="11">
+      <c r="K49">
         <v>13</v>
       </c>
       <c r="L49">
@@ -27310,10 +27313,10 @@
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="J50" s="11">
+      <c r="J50">
         <v>8</v>
       </c>
-      <c r="K50" s="11">
+      <c r="K50">
         <v>10</v>
       </c>
       <c r="L50">
@@ -27498,10 +27501,10 @@
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="J51" s="11">
+      <c r="J51">
         <v>8</v>
       </c>
-      <c r="K51" s="11">
+      <c r="K51">
         <v>8</v>
       </c>
       <c r="L51">
@@ -27686,10 +27689,10 @@
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J52" s="11">
+      <c r="J52">
         <v>8</v>
       </c>
-      <c r="K52" s="11">
+      <c r="K52">
         <v>10</v>
       </c>
       <c r="L52">
@@ -27874,10 +27877,10 @@
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="J53" s="11">
+      <c r="J53">
         <v>8</v>
       </c>
-      <c r="K53" s="11">
+      <c r="K53">
         <v>10</v>
       </c>
       <c r="L53">
@@ -28062,10 +28065,10 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="J54" s="11">
+      <c r="J54">
         <v>6</v>
       </c>
-      <c r="K54" s="11">
+      <c r="K54">
         <v>8</v>
       </c>
       <c r="L54">
@@ -28250,10 +28253,10 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="J55" s="11">
+      <c r="J55">
         <v>8</v>
       </c>
-      <c r="K55" s="11">
+      <c r="K55">
         <v>22</v>
       </c>
       <c r="L55">
@@ -28438,10 +28441,10 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J56" s="11">
-        <v>0</v>
-      </c>
-      <c r="K56" s="11">
+      <c r="J56">
+        <v>0</v>
+      </c>
+      <c r="K56">
         <v>0</v>
       </c>
       <c r="L56">
@@ -28626,10 +28629,10 @@
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J57" s="11">
+      <c r="J57">
         <v>8</v>
       </c>
-      <c r="K57" s="11">
+      <c r="K57">
         <v>13</v>
       </c>
       <c r="L57">
@@ -28814,10 +28817,10 @@
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="J58" s="11">
+      <c r="J58">
         <v>8</v>
       </c>
-      <c r="K58" s="11">
+      <c r="K58">
         <v>13</v>
       </c>
       <c r="L58">
@@ -29002,10 +29005,10 @@
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="J59" s="11">
+      <c r="J59">
         <v>6</v>
       </c>
-      <c r="K59" s="11">
+      <c r="K59">
         <v>8</v>
       </c>
       <c r="L59">
@@ -29190,10 +29193,10 @@
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="J60" s="11">
+      <c r="J60">
         <v>13</v>
       </c>
-      <c r="K60" s="11">
+      <c r="K60">
         <v>20</v>
       </c>
       <c r="L60">
@@ -29566,10 +29569,10 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="J62" s="11">
+      <c r="J62">
         <v>8</v>
       </c>
-      <c r="K62" s="11">
+      <c r="K62">
         <v>15</v>
       </c>
       <c r="L62">
@@ -29754,10 +29757,10 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="J63" s="11">
+      <c r="J63">
         <v>6</v>
       </c>
-      <c r="K63" s="11">
+      <c r="K63">
         <v>10</v>
       </c>
       <c r="L63">
@@ -29942,10 +29945,10 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="J64" s="11">
+      <c r="J64">
         <v>8</v>
       </c>
-      <c r="K64" s="11">
+      <c r="K64">
         <v>10</v>
       </c>
       <c r="L64">
@@ -30130,10 +30133,10 @@
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="J65" s="11">
+      <c r="J65">
         <v>8</v>
       </c>
-      <c r="K65" s="11">
+      <c r="K65">
         <v>22</v>
       </c>
       <c r="L65">
@@ -30318,10 +30321,10 @@
         <f t="shared" ref="I66:I78" si="3">SUM(L66:AO66)</f>
         <v>17</v>
       </c>
-      <c r="J66" s="11">
+      <c r="J66">
         <v>8</v>
       </c>
-      <c r="K66" s="11">
+      <c r="K66">
         <v>13</v>
       </c>
       <c r="L66">
@@ -30506,10 +30509,10 @@
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="J67" s="11">
+      <c r="J67">
         <v>6</v>
       </c>
-      <c r="K67" s="11">
+      <c r="K67">
         <v>10</v>
       </c>
       <c r="L67">
@@ -30694,10 +30697,10 @@
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="J68" s="11">
+      <c r="J68">
         <v>8</v>
       </c>
-      <c r="K68" s="11">
+      <c r="K68">
         <v>17</v>
       </c>
       <c r="L68">
@@ -30882,10 +30885,10 @@
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="J69" s="11">
+      <c r="J69">
         <v>6</v>
       </c>
-      <c r="K69" s="11">
+      <c r="K69">
         <v>20</v>
       </c>
       <c r="L69">
@@ -31070,10 +31073,10 @@
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="J70" s="11">
+      <c r="J70">
         <v>8</v>
       </c>
-      <c r="K70" s="11">
+      <c r="K70">
         <v>13</v>
       </c>
       <c r="L70">
@@ -31258,10 +31261,10 @@
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="J71" s="11">
+      <c r="J71">
         <v>10</v>
       </c>
-      <c r="K71" s="11">
+      <c r="K71">
         <v>22</v>
       </c>
       <c r="L71">
@@ -31446,10 +31449,10 @@
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="J72" s="11">
+      <c r="J72">
         <v>10</v>
       </c>
-      <c r="K72" s="11">
+      <c r="K72">
         <v>13</v>
       </c>
       <c r="L72">
@@ -31634,10 +31637,10 @@
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="J73" s="11">
+      <c r="J73">
         <v>8</v>
       </c>
-      <c r="K73" s="11">
+      <c r="K73">
         <v>10</v>
       </c>
       <c r="L73">
@@ -31822,10 +31825,10 @@
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="J74" s="11">
+      <c r="J74">
         <v>8</v>
       </c>
-      <c r="K74" s="11">
+      <c r="K74">
         <v>13</v>
       </c>
       <c r="L74">
@@ -32010,10 +32013,10 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="J75" s="11">
+      <c r="J75">
         <v>8</v>
       </c>
-      <c r="K75" s="11">
+      <c r="K75">
         <v>10</v>
       </c>
       <c r="L75">
@@ -32386,10 +32389,10 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J77" s="11">
-        <v>0</v>
-      </c>
-      <c r="K77" s="11">
+      <c r="J77">
+        <v>0</v>
+      </c>
+      <c r="K77">
         <v>0</v>
       </c>
       <c r="L77">
@@ -32574,10 +32577,10 @@
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="J78" s="11">
+      <c r="J78">
         <v>13</v>
       </c>
-      <c r="K78" s="11">
+      <c r="K78">
         <v>20</v>
       </c>
       <c r="L78">
@@ -32762,10 +32765,10 @@
         <f t="shared" ref="I79:I87" si="5">SUM(L79:AX79)</f>
         <v>13</v>
       </c>
-      <c r="J79" s="11">
+      <c r="J79">
         <v>13</v>
       </c>
-      <c r="K79" s="11">
+      <c r="K79">
         <v>29</v>
       </c>
       <c r="L79">
@@ -32949,10 +32952,10 @@
         <f t="shared" ref="I80:I86" si="6">SUM(L80:AX80)</f>
         <v>19</v>
       </c>
-      <c r="J80" s="11">
+      <c r="J80">
         <v>13</v>
       </c>
-      <c r="K80" s="11">
+      <c r="K80">
         <v>20</v>
       </c>
       <c r="L80">
@@ -33136,10 +33139,10 @@
         <f t="shared" si="6"/>
         <v>20</v>
       </c>
-      <c r="J81" s="11">
+      <c r="J81">
         <v>10</v>
       </c>
-      <c r="K81" s="11">
+      <c r="K81">
         <v>13</v>
       </c>
       <c r="L81">
@@ -33323,10 +33326,10 @@
         <f t="shared" si="6"/>
         <v>12</v>
       </c>
-      <c r="J82" s="11">
+      <c r="J82">
         <v>13</v>
       </c>
-      <c r="K82" s="11">
+      <c r="K82">
         <v>15</v>
       </c>
       <c r="L82">
@@ -33510,10 +33513,10 @@
         <f t="shared" si="6"/>
         <v>18</v>
       </c>
-      <c r="J83" s="11">
+      <c r="J83">
         <v>10</v>
       </c>
-      <c r="K83" s="11">
+      <c r="K83">
         <v>15</v>
       </c>
       <c r="L83">
@@ -33697,10 +33700,10 @@
         <f t="shared" si="6"/>
         <v>20</v>
       </c>
-      <c r="J84" s="11">
+      <c r="J84">
         <v>10</v>
       </c>
-      <c r="K84" s="11">
+      <c r="K84">
         <v>13</v>
       </c>
       <c r="L84">
@@ -33884,10 +33887,10 @@
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="J85" s="11">
+      <c r="J85">
         <v>10</v>
       </c>
-      <c r="K85" s="11">
+      <c r="K85">
         <v>10</v>
       </c>
       <c r="L85">
@@ -34071,10 +34074,10 @@
         <f t="shared" si="6"/>
         <v>17</v>
       </c>
-      <c r="J86" s="11">
+      <c r="J86">
         <v>13</v>
       </c>
-      <c r="K86" s="11">
+      <c r="K86">
         <v>17</v>
       </c>
       <c r="L86">
@@ -34258,10 +34261,10 @@
         <f t="shared" si="5"/>
         <v>14</v>
       </c>
-      <c r="J87" s="11">
+      <c r="J87">
         <v>10</v>
       </c>
-      <c r="K87" s="11">
+      <c r="K87">
         <v>24</v>
       </c>
       <c r="L87">
@@ -34445,10 +34448,10 @@
         <f>SUM(L88:AO88)</f>
         <v>17</v>
       </c>
-      <c r="J88" s="11">
+      <c r="J88">
         <v>10</v>
       </c>
-      <c r="K88" s="11">
+      <c r="K88">
         <v>13</v>
       </c>
       <c r="L88">
@@ -34632,10 +34635,10 @@
         <f>SUM(L89:AO89)</f>
         <v>18</v>
       </c>
-      <c r="J89" s="11">
+      <c r="J89">
         <v>10</v>
       </c>
-      <c r="K89" s="11">
+      <c r="K89">
         <v>17</v>
       </c>
       <c r="L89">
@@ -34819,10 +34822,10 @@
         <f>SUM(L90:AO90)</f>
         <v>1</v>
       </c>
-      <c r="J90" s="11">
+      <c r="J90">
         <v>20</v>
       </c>
-      <c r="K90" s="11">
+      <c r="K90">
         <v>20</v>
       </c>
       <c r="L90">
@@ -35006,10 +35009,10 @@
         <f>SUM(L91:AO91)</f>
         <v>18</v>
       </c>
-      <c r="J91" s="11">
+      <c r="J91">
         <v>10</v>
       </c>
-      <c r="K91" s="11">
+      <c r="K91">
         <v>20</v>
       </c>
       <c r="L91">
@@ -35386,7 +35389,7 @@
         <v>0.64</v>
       </c>
       <c r="F2" s="2">
-        <f>(I2+G2)/20</f>
+        <f t="shared" ref="F2:F33" si="0">(I2+G2)/20</f>
         <v>0.05</v>
       </c>
       <c r="G2" s="2">
@@ -35396,7 +35399,7 @@
         <v>20</v>
       </c>
       <c r="I2" s="2">
-        <f t="shared" ref="I2:I16" si="0">SUM(L2:AV2)</f>
+        <f t="shared" ref="I2:I16" si="1">SUM(L2:AV2)</f>
         <v>1</v>
       </c>
       <c r="J2" s="2">
@@ -35573,7 +35576,7 @@
         <v>0.87</v>
       </c>
       <c r="F3">
-        <f>(I3+G3)/20</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G3">
@@ -35583,7 +35586,7 @@
         <v>20</v>
       </c>
       <c r="I3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="J3">
@@ -35761,7 +35764,7 @@
         <v>0.82</v>
       </c>
       <c r="F4">
-        <f>(I4+G4)/20</f>
+        <f t="shared" si="0"/>
         <v>0.95</v>
       </c>
       <c r="G4">
@@ -35771,7 +35774,7 @@
         <v>20</v>
       </c>
       <c r="I4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="J4">
@@ -35949,7 +35952,7 @@
         <v>0.89</v>
       </c>
       <c r="F5">
-        <f>(I5+G5)/20</f>
+        <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
       <c r="G5">
@@ -35959,7 +35962,7 @@
         <v>20</v>
       </c>
       <c r="I5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="J5">
@@ -36137,7 +36140,7 @@
         <v>0.92</v>
       </c>
       <c r="F6">
-        <f>(I6+G6)/20</f>
+        <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
       <c r="G6">
@@ -36147,7 +36150,7 @@
         <v>20</v>
       </c>
       <c r="I6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="J6">
@@ -36325,7 +36328,7 @@
         <v>0.95</v>
       </c>
       <c r="F7">
-        <f>(I7+G7)/20</f>
+        <f t="shared" si="0"/>
         <v>0.65</v>
       </c>
       <c r="G7">
@@ -36335,7 +36338,7 @@
         <v>20</v>
       </c>
       <c r="I7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="J7">
@@ -36513,7 +36516,7 @@
         <v>0.93</v>
       </c>
       <c r="F8">
-        <f>(I8+G8)/20</f>
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="G8">
@@ -36523,7 +36526,7 @@
         <v>20</v>
       </c>
       <c r="I8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="J8">
@@ -36701,7 +36704,7 @@
         <v>0.93</v>
       </c>
       <c r="F9">
-        <f>(I9+G9)/20</f>
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
       <c r="G9">
@@ -36711,7 +36714,7 @@
         <v>20</v>
       </c>
       <c r="I9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="J9">
@@ -36889,7 +36892,7 @@
         <v>0.93</v>
       </c>
       <c r="F10">
-        <f>(I10+G10)/20</f>
+        <f t="shared" si="0"/>
         <v>0.7</v>
       </c>
       <c r="G10">
@@ -36899,7 +36902,7 @@
         <v>20</v>
       </c>
       <c r="I10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="J10">
@@ -37077,7 +37080,7 @@
         <v>0.93</v>
       </c>
       <c r="F11">
-        <f>(I11+G11)/20</f>
+        <f t="shared" si="0"/>
         <v>0.85</v>
       </c>
       <c r="G11">
@@ -37087,7 +37090,7 @@
         <v>20</v>
       </c>
       <c r="I11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="J11">
@@ -37265,7 +37268,7 @@
         <v>0.85</v>
       </c>
       <c r="F12">
-        <f>(I12+G12)/20</f>
+        <f t="shared" si="0"/>
         <v>0.95</v>
       </c>
       <c r="G12">
@@ -37275,7 +37278,7 @@
         <v>20</v>
       </c>
       <c r="I12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="J12">
@@ -37453,7 +37456,7 @@
         <v>0.8</v>
       </c>
       <c r="F13">
-        <f>(I13+G13)/20</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G13">
@@ -37463,7 +37466,7 @@
         <v>20</v>
       </c>
       <c r="I13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="J13">
@@ -37641,7 +37644,7 @@
         <v>0.92</v>
       </c>
       <c r="F14">
-        <f>(I14+G14)/20</f>
+        <f t="shared" si="0"/>
         <v>0.85</v>
       </c>
       <c r="G14">
@@ -37651,7 +37654,7 @@
         <v>20</v>
       </c>
       <c r="I14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="J14">
@@ -37829,7 +37832,7 @@
         <v>0.86</v>
       </c>
       <c r="F15">
-        <f>(I15+G15)/20</f>
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
       <c r="G15">
@@ -37839,7 +37842,7 @@
         <v>20</v>
       </c>
       <c r="I15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="J15">
@@ -38017,7 +38020,7 @@
         <v>0.91</v>
       </c>
       <c r="F16" s="6">
-        <f>(I16+G16)/20</f>
+        <f t="shared" si="0"/>
         <v>0.7</v>
       </c>
       <c r="G16" s="6">
@@ -38027,7 +38030,7 @@
         <v>20</v>
       </c>
       <c r="I16" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="J16" s="6">
@@ -38205,7 +38208,7 @@
         <v>0.67</v>
       </c>
       <c r="F17">
-        <f>(I17+G17)/20</f>
+        <f t="shared" si="0"/>
         <v>0.65</v>
       </c>
       <c r="G17">
@@ -38215,13 +38218,13 @@
         <v>20</v>
       </c>
       <c r="I17">
-        <f t="shared" ref="I17:I67" si="1">SUM(L17:BA17)</f>
+        <f t="shared" ref="I17:I67" si="2">SUM(L17:BA17)</f>
         <v>11</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17">
         <v>8</v>
       </c>
-      <c r="K17" s="11">
+      <c r="K17">
         <v>13</v>
       </c>
       <c r="L17">
@@ -38393,7 +38396,7 @@
         <v>0.82</v>
       </c>
       <c r="F18">
-        <f>(I18+G18)/20</f>
+        <f t="shared" si="0"/>
         <v>0.65</v>
       </c>
       <c r="G18">
@@ -38403,13 +38406,13 @@
         <v>20</v>
       </c>
       <c r="I18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18">
         <v>6</v>
       </c>
-      <c r="K18" s="11">
+      <c r="K18">
         <v>8</v>
       </c>
       <c r="L18">
@@ -38581,7 +38584,7 @@
         <v>0.87</v>
       </c>
       <c r="F19">
-        <f>(I19+G19)/20</f>
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="G19">
@@ -38591,13 +38594,13 @@
         <v>20</v>
       </c>
       <c r="I19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19">
         <v>8</v>
       </c>
-      <c r="K19" s="11">
+      <c r="K19">
         <v>13</v>
       </c>
       <c r="L19">
@@ -38769,7 +38772,7 @@
         <v>0.82</v>
       </c>
       <c r="F20">
-        <f>(I20+G20)/20</f>
+        <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
       <c r="G20">
@@ -38779,13 +38782,13 @@
         <v>20</v>
       </c>
       <c r="I20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20">
         <v>8</v>
       </c>
-      <c r="K20" s="11">
+      <c r="K20">
         <v>8</v>
       </c>
       <c r="L20">
@@ -38957,7 +38960,7 @@
         <v>0.93</v>
       </c>
       <c r="F21">
-        <f>(I21+G21)/20</f>
+        <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
       <c r="G21">
@@ -38967,13 +38970,13 @@
         <v>20</v>
       </c>
       <c r="I21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21">
         <v>8</v>
       </c>
-      <c r="K21" s="11">
+      <c r="K21">
         <v>8</v>
       </c>
       <c r="L21">
@@ -39145,7 +39148,7 @@
         <v>0.95</v>
       </c>
       <c r="F22">
-        <f>(I22+G22)/20</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G22">
@@ -39155,13 +39158,13 @@
         <v>20</v>
       </c>
       <c r="I22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22">
         <v>6</v>
       </c>
-      <c r="K22" s="11">
+      <c r="K22">
         <v>10</v>
       </c>
       <c r="L22">
@@ -39333,7 +39336,7 @@
         <v>0.93</v>
       </c>
       <c r="F23">
-        <f>(I23+G23)/20</f>
+        <f t="shared" si="0"/>
         <v>0.85</v>
       </c>
       <c r="G23">
@@ -39343,13 +39346,13 @@
         <v>20</v>
       </c>
       <c r="I23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J23" s="11">
+      <c r="J23">
         <v>8</v>
       </c>
-      <c r="K23" s="11">
+      <c r="K23">
         <v>13</v>
       </c>
       <c r="L23">
@@ -39521,7 +39524,7 @@
         <v>0.93</v>
       </c>
       <c r="F24">
-        <f>(I24+G24)/20</f>
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
       <c r="G24">
@@ -39531,13 +39534,13 @@
         <v>20</v>
       </c>
       <c r="I24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J24" s="11">
+      <c r="J24">
         <v>8</v>
       </c>
-      <c r="K24" s="11">
+      <c r="K24">
         <v>13</v>
       </c>
       <c r="L24">
@@ -39709,7 +39712,7 @@
         <v>0.93</v>
       </c>
       <c r="F25">
-        <f>(I25+G25)/20</f>
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
       <c r="G25">
@@ -39719,13 +39722,13 @@
         <v>20</v>
       </c>
       <c r="I25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J25" s="11">
+      <c r="J25">
         <v>8</v>
       </c>
-      <c r="K25" s="11">
+      <c r="K25">
         <v>10</v>
       </c>
       <c r="L25">
@@ -39897,7 +39900,7 @@
         <v>0.85</v>
       </c>
       <c r="F26">
-        <f>(I26+G26)/20</f>
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
       <c r="G26">
@@ -39907,13 +39910,13 @@
         <v>20</v>
       </c>
       <c r="I26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J26" s="11">
+      <c r="J26">
         <v>8</v>
       </c>
-      <c r="K26" s="11">
+      <c r="K26">
         <v>8</v>
       </c>
       <c r="L26">
@@ -40085,7 +40088,7 @@
         <v>0.96</v>
       </c>
       <c r="F27">
-        <f>(I27+G27)/20</f>
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
       <c r="G27">
@@ -40095,13 +40098,13 @@
         <v>20</v>
       </c>
       <c r="I27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J27" s="11">
+      <c r="J27">
         <v>6</v>
       </c>
-      <c r="K27" s="11">
+      <c r="K27">
         <v>13</v>
       </c>
       <c r="L27">
@@ -40273,7 +40276,7 @@
         <v>0.83</v>
       </c>
       <c r="F28">
-        <f>(I28+G28)/20</f>
+        <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
       <c r="G28">
@@ -40283,13 +40286,13 @@
         <v>20</v>
       </c>
       <c r="I28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="J28" s="11">
+      <c r="J28">
         <v>8</v>
       </c>
-      <c r="K28" s="11">
+      <c r="K28">
         <v>8</v>
       </c>
       <c r="L28">
@@ -40461,7 +40464,7 @@
         <v>0.52</v>
       </c>
       <c r="F29">
-        <f>(I29+G29)/20</f>
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
       <c r="G29">
@@ -40471,13 +40474,13 @@
         <v>20</v>
       </c>
       <c r="I29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J29">
         <v>6</v>
       </c>
-      <c r="K29" s="11">
+      <c r="K29">
         <v>8</v>
       </c>
       <c r="L29">
@@ -40649,7 +40652,7 @@
         <v>0.8</v>
       </c>
       <c r="F30">
-        <f>(I30+G30)/20</f>
+        <f t="shared" si="0"/>
         <v>0.65</v>
       </c>
       <c r="G30">
@@ -40659,13 +40662,13 @@
         <v>20</v>
       </c>
       <c r="I30">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30">
         <v>8</v>
       </c>
-      <c r="K30" s="11">
+      <c r="K30">
         <v>10</v>
       </c>
       <c r="L30">
@@ -40837,7 +40840,7 @@
         <v>0.89</v>
       </c>
       <c r="F31" s="6">
-        <f>(I31+G31)/20</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G31" s="6">
@@ -40847,7 +40850,7 @@
         <v>20</v>
       </c>
       <c r="I31" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J31" s="6">
@@ -41025,7 +41028,7 @@
         <v>0.67</v>
       </c>
       <c r="F32">
-        <f>(I32+G32)/20</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="G32">
@@ -41035,13 +41038,13 @@
         <v>20</v>
       </c>
       <c r="I32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="J32" s="11">
+      <c r="J32">
         <v>10</v>
       </c>
-      <c r="K32" s="11">
+      <c r="K32">
         <v>13</v>
       </c>
       <c r="L32">
@@ -41213,7 +41216,7 @@
         <v>0.87</v>
       </c>
       <c r="F33">
-        <f>(I33+G33)/20</f>
+        <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
       <c r="G33">
@@ -41223,13 +41226,13 @@
         <v>20</v>
       </c>
       <c r="I33">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J33">
         <v>13</v>
       </c>
-      <c r="K33" s="11">
+      <c r="K33">
         <v>15</v>
       </c>
       <c r="L33">
@@ -41401,7 +41404,7 @@
         <v>0.92</v>
       </c>
       <c r="F34">
-        <f>(I34+G34)/20</f>
+        <f t="shared" ref="F34:F65" si="3">(I34+G34)/20</f>
         <v>0.8</v>
       </c>
       <c r="G34">
@@ -41411,13 +41414,13 @@
         <v>20</v>
       </c>
       <c r="I34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="J34" s="11">
+      <c r="J34">
         <v>13</v>
       </c>
-      <c r="K34" s="11">
+      <c r="K34">
         <v>13</v>
       </c>
       <c r="L34">
@@ -41589,7 +41592,7 @@
         <v>0.93</v>
       </c>
       <c r="F35">
-        <f>(I35+G35)/20</f>
+        <f t="shared" si="3"/>
         <v>0.75</v>
       </c>
       <c r="G35">
@@ -41599,13 +41602,13 @@
         <v>20</v>
       </c>
       <c r="I35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="J35" s="11">
+      <c r="J35">
         <v>10</v>
       </c>
-      <c r="K35" s="11">
+      <c r="K35">
         <v>15</v>
       </c>
       <c r="L35">
@@ -41777,7 +41780,7 @@
         <v>0.95</v>
       </c>
       <c r="F36">
-        <f>(I36+G36)/20</f>
+        <f t="shared" si="3"/>
         <v>0.95</v>
       </c>
       <c r="G36">
@@ -41787,13 +41790,13 @@
         <v>20</v>
       </c>
       <c r="I36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="J36" s="11">
+      <c r="J36">
         <v>10</v>
       </c>
-      <c r="K36" s="11">
+      <c r="K36">
         <v>15</v>
       </c>
       <c r="L36">
@@ -41965,7 +41968,7 @@
         <v>0.93</v>
       </c>
       <c r="F37">
-        <f>(I37+G37)/20</f>
+        <f t="shared" si="3"/>
         <v>0.85</v>
       </c>
       <c r="G37">
@@ -41975,13 +41978,13 @@
         <v>20</v>
       </c>
       <c r="I37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J37" s="11">
+      <c r="J37">
         <v>13</v>
       </c>
-      <c r="K37" s="11">
+      <c r="K37">
         <v>15</v>
       </c>
       <c r="L37">
@@ -42153,7 +42156,7 @@
         <v>0.93</v>
       </c>
       <c r="F38">
-        <f>(I38+G38)/20</f>
+        <f t="shared" si="3"/>
         <v>0.95</v>
       </c>
       <c r="G38">
@@ -42163,13 +42166,13 @@
         <v>20</v>
       </c>
       <c r="I38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="J38" s="11">
+      <c r="J38">
         <v>10</v>
       </c>
-      <c r="K38" s="11">
+      <c r="K38">
         <v>13</v>
       </c>
       <c r="L38">
@@ -42341,7 +42344,7 @@
         <v>0.93</v>
       </c>
       <c r="F39">
-        <f>(I39+G39)/20</f>
+        <f t="shared" si="3"/>
         <v>0.85</v>
       </c>
       <c r="G39">
@@ -42351,13 +42354,13 @@
         <v>20</v>
       </c>
       <c r="I39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J39" s="11">
+      <c r="J39">
         <v>13</v>
       </c>
-      <c r="K39" s="11">
+      <c r="K39">
         <v>29</v>
       </c>
       <c r="L39">
@@ -42528,7 +42531,7 @@
         <v>0.93</v>
       </c>
       <c r="F40">
-        <f>(I40+G40)/20</f>
+        <f t="shared" si="3"/>
         <v>0.9</v>
       </c>
       <c r="G40">
@@ -42538,13 +42541,13 @@
         <v>20</v>
       </c>
       <c r="I40">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J40" s="11">
+      <c r="J40">
         <v>10</v>
       </c>
-      <c r="K40" s="11">
+      <c r="K40">
         <v>29</v>
       </c>
       <c r="L40">
@@ -42715,7 +42718,7 @@
         <v>0.85</v>
       </c>
       <c r="F41">
-        <f>(I41+G41)/20</f>
+        <f t="shared" si="3"/>
         <v>0.9</v>
       </c>
       <c r="G41">
@@ -42725,13 +42728,13 @@
         <v>20</v>
       </c>
       <c r="I41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J41" s="11">
+      <c r="J41">
         <v>13</v>
       </c>
-      <c r="K41" s="11">
+      <c r="K41">
         <v>20</v>
       </c>
       <c r="L41">
@@ -42902,7 +42905,7 @@
         <v>0.96</v>
       </c>
       <c r="F42">
-        <f>(I42+G42)/20</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G42">
@@ -42912,13 +42915,13 @@
         <v>20</v>
       </c>
       <c r="I42">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="J42" s="11">
+      <c r="J42">
         <v>10</v>
       </c>
-      <c r="K42" s="11">
+      <c r="K42">
         <v>13</v>
       </c>
       <c r="L42">
@@ -43089,7 +43092,7 @@
         <v>0.65</v>
       </c>
       <c r="F43">
-        <f>(I43+G43)/20</f>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="G43">
@@ -43099,13 +43102,13 @@
         <v>20</v>
       </c>
       <c r="I43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="J43" s="11">
+      <c r="J43">
         <v>10</v>
       </c>
-      <c r="K43" s="11">
+      <c r="K43">
         <v>13</v>
       </c>
       <c r="L43">
@@ -43276,7 +43279,7 @@
         <v>0.52</v>
       </c>
       <c r="F44">
-        <f>(I44+G44)/20</f>
+        <f t="shared" si="3"/>
         <v>0.65</v>
       </c>
       <c r="G44">
@@ -43286,13 +43289,13 @@
         <v>20</v>
       </c>
       <c r="I44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="J44" s="11">
+      <c r="J44">
         <v>10</v>
       </c>
-      <c r="K44" s="11">
+      <c r="K44">
         <v>15</v>
       </c>
       <c r="L44">
@@ -43463,7 +43466,7 @@
         <v>0.8</v>
       </c>
       <c r="F45">
-        <f>(I45+G45)/20</f>
+        <f t="shared" si="3"/>
         <v>0.8</v>
       </c>
       <c r="G45">
@@ -43473,13 +43476,13 @@
         <v>20</v>
       </c>
       <c r="I45">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="J45" s="11">
+      <c r="J45">
         <v>10</v>
       </c>
-      <c r="K45" s="11">
+      <c r="K45">
         <v>24</v>
       </c>
       <c r="L45">
@@ -43650,7 +43653,7 @@
         <v>0.92</v>
       </c>
       <c r="F46" s="6">
-        <f>(I46+G46)/20</f>
+        <f t="shared" si="3"/>
         <v>0.85</v>
       </c>
       <c r="G46" s="6">
@@ -43660,7 +43663,7 @@
         <v>20</v>
       </c>
       <c r="I46" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
       <c r="J46" s="6">
@@ -43837,7 +43840,7 @@
         <v>0.84</v>
       </c>
       <c r="F47">
-        <f>(I47+G47)/20</f>
+        <f t="shared" si="3"/>
         <v>0.75</v>
       </c>
       <c r="G47">
@@ -43847,13 +43850,13 @@
         <v>20</v>
       </c>
       <c r="I47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="J47" s="11">
+      <c r="J47">
         <v>8</v>
       </c>
-      <c r="K47" s="11">
+      <c r="K47">
         <v>10</v>
       </c>
       <c r="L47">
@@ -44024,7 +44027,7 @@
         <v>0.92</v>
       </c>
       <c r="F48">
-        <f>(I48+G48)/20</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G48">
@@ -44034,13 +44037,13 @@
         <v>20</v>
       </c>
       <c r="I48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="J48" s="11">
+      <c r="J48">
         <v>6</v>
       </c>
-      <c r="K48" s="11">
+      <c r="K48">
         <v>8</v>
       </c>
       <c r="L48">
@@ -44211,7 +44214,7 @@
         <v>0.87</v>
       </c>
       <c r="F49">
-        <f>(I49+G49)/20</f>
+        <f t="shared" si="3"/>
         <v>0.85</v>
       </c>
       <c r="G49">
@@ -44221,13 +44224,13 @@
         <v>20</v>
       </c>
       <c r="I49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J49" s="11">
+      <c r="J49">
         <v>8</v>
       </c>
-      <c r="K49" s="11">
+      <c r="K49">
         <v>8</v>
       </c>
       <c r="L49">
@@ -44398,7 +44401,7 @@
         <v>0.74</v>
       </c>
       <c r="F50">
-        <f>(I50+G50)/20</f>
+        <f t="shared" si="3"/>
         <v>0.65</v>
       </c>
       <c r="G50">
@@ -44408,13 +44411,13 @@
         <v>20</v>
       </c>
       <c r="I50">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="J50" s="11">
+      <c r="J50">
         <v>6</v>
       </c>
-      <c r="K50" s="11">
+      <c r="K50">
         <v>10</v>
       </c>
       <c r="L50">
@@ -44585,7 +44588,7 @@
         <v>0.64</v>
       </c>
       <c r="F51">
-        <f>(I51+G51)/20</f>
+        <f t="shared" si="3"/>
         <v>0.25</v>
       </c>
       <c r="G51">
@@ -44595,13 +44598,13 @@
         <v>20</v>
       </c>
       <c r="I51">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="J51" s="11">
+      <c r="J51">
         <v>13</v>
       </c>
-      <c r="K51" s="11">
+      <c r="K51">
         <v>20</v>
       </c>
       <c r="L51">
@@ -44772,7 +44775,7 @@
         <v>0.82</v>
       </c>
       <c r="F52">
-        <f>(I52+G52)/20</f>
+        <f t="shared" si="3"/>
         <v>0.85</v>
       </c>
       <c r="G52">
@@ -44782,13 +44785,13 @@
         <v>20</v>
       </c>
       <c r="I52">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J52" s="11">
+      <c r="J52">
         <v>8</v>
       </c>
-      <c r="K52" s="11">
+      <c r="K52">
         <v>13</v>
       </c>
       <c r="L52">
@@ -44959,7 +44962,7 @@
         <v>0.89</v>
       </c>
       <c r="F53">
-        <f>(I53+G53)/20</f>
+        <f t="shared" si="3"/>
         <v>0.7</v>
       </c>
       <c r="G53">
@@ -44969,13 +44972,13 @@
         <v>20</v>
       </c>
       <c r="I53">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="J53" s="11">
+      <c r="J53">
         <v>10</v>
       </c>
-      <c r="K53" s="11">
+      <c r="K53">
         <v>22</v>
       </c>
       <c r="L53">
@@ -45146,7 +45149,7 @@
         <v>0.93</v>
       </c>
       <c r="F54">
-        <f>(I54+G54)/20</f>
+        <f t="shared" si="3"/>
         <v>0.75</v>
       </c>
       <c r="G54">
@@ -45156,13 +45159,13 @@
         <v>20</v>
       </c>
       <c r="I54">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="J54" s="11">
+      <c r="J54">
         <v>8</v>
       </c>
-      <c r="K54" s="11">
+      <c r="K54">
         <v>13</v>
       </c>
       <c r="L54">
@@ -45333,7 +45336,7 @@
         <v>0.95</v>
       </c>
       <c r="F55">
-        <f>(I55+G55)/20</f>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="G55">
@@ -45343,13 +45346,13 @@
         <v>20</v>
       </c>
       <c r="I55">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="J55" s="11">
+      <c r="J55">
         <v>8</v>
       </c>
-      <c r="K55" s="11">
+      <c r="K55">
         <v>10</v>
       </c>
       <c r="L55">
@@ -45520,7 +45523,7 @@
         <v>0.93</v>
       </c>
       <c r="F56">
-        <f>(I56+G56)/20</f>
+        <f t="shared" si="3"/>
         <v>0.9</v>
       </c>
       <c r="G56">
@@ -45530,13 +45533,13 @@
         <v>20</v>
       </c>
       <c r="I56">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="J56" s="11">
+      <c r="J56">
         <v>8</v>
       </c>
-      <c r="K56" s="11">
+      <c r="K56">
         <v>13</v>
       </c>
       <c r="L56">
@@ -45707,7 +45710,7 @@
         <v>0.85</v>
       </c>
       <c r="F57">
-        <f>(I57+G57)/20</f>
+        <f t="shared" si="3"/>
         <v>0.7</v>
       </c>
       <c r="G57">
@@ -45717,13 +45720,13 @@
         <v>20</v>
       </c>
       <c r="I57">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="J57" s="11">
+      <c r="J57">
         <v>8</v>
       </c>
-      <c r="K57" s="11">
+      <c r="K57">
         <v>17</v>
       </c>
       <c r="L57">
@@ -45894,7 +45897,7 @@
         <v>0.83</v>
       </c>
       <c r="F58">
-        <f>(I58+G58)/20</f>
+        <f t="shared" si="3"/>
         <v>0.75</v>
       </c>
       <c r="G58">
@@ -45904,13 +45907,13 @@
         <v>20</v>
       </c>
       <c r="I58">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="J58" s="11">
+      <c r="J58">
         <v>8</v>
       </c>
-      <c r="K58" s="11">
+      <c r="K58">
         <v>15</v>
       </c>
       <c r="L58">
@@ -46081,7 +46084,7 @@
         <v>0.52</v>
       </c>
       <c r="F59">
-        <f>(I59+G59)/20</f>
+        <f t="shared" si="3"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="G59">
@@ -46091,13 +46094,13 @@
         <v>20</v>
       </c>
       <c r="I59">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="J59" s="11">
+      <c r="J59">
         <v>8</v>
       </c>
-      <c r="K59" s="11">
+      <c r="K59">
         <v>13</v>
       </c>
       <c r="L59">
@@ -46268,7 +46271,7 @@
         <v>0.92</v>
       </c>
       <c r="F60">
-        <f>(I60+G60)/20</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G60">
@@ -46278,13 +46281,13 @@
         <v>20</v>
       </c>
       <c r="I60">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="J60" s="11">
+      <c r="J60">
         <v>8</v>
       </c>
-      <c r="K60" s="11">
+      <c r="K60">
         <v>13</v>
       </c>
       <c r="L60">
@@ -46455,7 +46458,7 @@
         <v>0.86</v>
       </c>
       <c r="F61" s="6">
-        <f>(I61+G61)/20</f>
+        <f t="shared" si="3"/>
         <v>0.8</v>
       </c>
       <c r="G61" s="6">
@@ -46465,7 +46468,7 @@
         <v>20</v>
       </c>
       <c r="I61" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
       <c r="J61" s="6">
@@ -46642,7 +46645,7 @@
         <v>0.67</v>
       </c>
       <c r="F62">
-        <f>(I62+G62)/20</f>
+        <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
       <c r="G62">
@@ -46652,13 +46655,13 @@
         <v>20</v>
       </c>
       <c r="I62">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="J62" s="11">
+      <c r="J62">
         <v>13</v>
       </c>
-      <c r="K62" s="11">
+      <c r="K62">
         <v>24</v>
       </c>
       <c r="L62">
@@ -46829,7 +46832,7 @@
         <v>0.82</v>
       </c>
       <c r="F63">
-        <f>(I63+G63)/20</f>
+        <f t="shared" si="3"/>
         <v>0.85</v>
       </c>
       <c r="G63">
@@ -46839,13 +46842,13 @@
         <v>20</v>
       </c>
       <c r="I63">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J63" s="11">
+      <c r="J63">
         <v>8</v>
       </c>
-      <c r="K63" s="11">
+      <c r="K63">
         <v>17</v>
       </c>
       <c r="L63">
@@ -47016,7 +47019,7 @@
         <v>0.74</v>
       </c>
       <c r="F64">
-        <f>(I64+G64)/20</f>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="G64">
@@ -47026,13 +47029,13 @@
         <v>20</v>
       </c>
       <c r="I64">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="J64" s="11">
+      <c r="J64">
         <v>8</v>
       </c>
-      <c r="K64" s="11">
+      <c r="K64">
         <v>8</v>
       </c>
       <c r="L64">
@@ -47203,7 +47206,7 @@
         <v>0.87</v>
       </c>
       <c r="F65">
-        <f>(I65+G65)/20</f>
+        <f t="shared" si="3"/>
         <v>0.35</v>
       </c>
       <c r="G65">
@@ -47213,13 +47216,13 @@
         <v>20</v>
       </c>
       <c r="I65">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="J65" s="11">
+      <c r="J65">
         <v>8</v>
       </c>
-      <c r="K65" s="11">
+      <c r="K65">
         <v>10</v>
       </c>
       <c r="L65">
@@ -47390,7 +47393,7 @@
         <v>0.89</v>
       </c>
       <c r="F66">
-        <f>(I66+G66)/20</f>
+        <f t="shared" ref="F66:F97" si="4">(I66+G66)/20</f>
         <v>0.85</v>
       </c>
       <c r="G66">
@@ -47400,13 +47403,13 @@
         <v>20</v>
       </c>
       <c r="I66">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J66" s="11">
+      <c r="J66">
         <v>8</v>
       </c>
-      <c r="K66" s="11">
+      <c r="K66">
         <v>13</v>
       </c>
       <c r="L66">
@@ -47577,7 +47580,7 @@
         <v>0.93</v>
       </c>
       <c r="F67">
-        <f>(I67+G67)/20</f>
+        <f t="shared" si="4"/>
         <v>0.85</v>
       </c>
       <c r="G67">
@@ -47587,13 +47590,13 @@
         <v>20</v>
       </c>
       <c r="I67">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="J67" s="11">
+      <c r="J67">
         <v>10</v>
       </c>
-      <c r="K67" s="11">
+      <c r="K67">
         <v>29</v>
       </c>
       <c r="L67">
@@ -47764,7 +47767,7 @@
         <v>0.95</v>
       </c>
       <c r="F68">
-        <f>(I68+G68)/20</f>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="G68">
@@ -47774,13 +47777,13 @@
         <v>20</v>
       </c>
       <c r="I68">
-        <f t="shared" ref="I68:I91" si="2">SUM(L68:BA68)</f>
+        <f t="shared" ref="I68:I91" si="5">SUM(L68:BA68)</f>
         <v>19</v>
       </c>
-      <c r="J68" s="11">
+      <c r="J68">
         <v>8</v>
       </c>
-      <c r="K68" s="11">
+      <c r="K68">
         <v>13</v>
       </c>
       <c r="L68">
@@ -47951,7 +47954,7 @@
         <v>0.93</v>
       </c>
       <c r="F69">
-        <f>(I69+G69)/20</f>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="G69">
@@ -47961,13 +47964,13 @@
         <v>20</v>
       </c>
       <c r="I69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="J69" s="11">
+      <c r="J69">
         <v>10</v>
       </c>
-      <c r="K69" s="11">
+      <c r="K69">
         <v>20</v>
       </c>
       <c r="L69">
@@ -48138,7 +48141,7 @@
         <v>0.93</v>
       </c>
       <c r="F70">
-        <f>(I70+G70)/20</f>
+        <f t="shared" si="4"/>
         <v>0.35</v>
       </c>
       <c r="G70">
@@ -48148,13 +48151,13 @@
         <v>20</v>
       </c>
       <c r="I70">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>7</v>
       </c>
-      <c r="J70" s="11">
+      <c r="J70">
         <v>8</v>
       </c>
-      <c r="K70" s="11">
+      <c r="K70">
         <v>10</v>
       </c>
       <c r="L70">
@@ -48325,7 +48328,7 @@
         <v>0.85</v>
       </c>
       <c r="F71">
-        <f>(I71+G71)/20</f>
+        <f t="shared" si="4"/>
         <v>0.8</v>
       </c>
       <c r="G71">
@@ -48335,13 +48338,13 @@
         <v>20</v>
       </c>
       <c r="I71">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="J71" s="11">
+      <c r="J71">
         <v>8</v>
       </c>
-      <c r="K71" s="11">
+      <c r="K71">
         <v>13</v>
       </c>
       <c r="L71">
@@ -48512,7 +48515,7 @@
         <v>0.83</v>
       </c>
       <c r="F72">
-        <f>(I72+G72)/20</f>
+        <f t="shared" si="4"/>
         <v>0.85</v>
       </c>
       <c r="G72">
@@ -48522,13 +48525,13 @@
         <v>20</v>
       </c>
       <c r="I72">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>17</v>
       </c>
-      <c r="J72" s="11">
+      <c r="J72">
         <v>10</v>
       </c>
-      <c r="K72" s="11">
+      <c r="K72">
         <v>17</v>
       </c>
       <c r="L72">
@@ -48699,7 +48702,7 @@
         <v>0.52</v>
       </c>
       <c r="F73">
-        <f>(I73+G73)/20</f>
+        <f t="shared" si="4"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="G73">
@@ -48709,13 +48712,13 @@
         <v>20</v>
       </c>
       <c r="I73">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>11</v>
       </c>
-      <c r="J73" s="11">
+      <c r="J73">
         <v>8</v>
       </c>
-      <c r="K73" s="11">
+      <c r="K73">
         <v>13</v>
       </c>
       <c r="L73">
@@ -48886,7 +48889,7 @@
         <v>0.8</v>
       </c>
       <c r="F74">
-        <f>(I74+G74)/20</f>
+        <f t="shared" si="4"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="G74">
@@ -48896,13 +48899,13 @@
         <v>20</v>
       </c>
       <c r="I74">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>11</v>
       </c>
-      <c r="J74" s="11">
+      <c r="J74">
         <v>8</v>
       </c>
-      <c r="K74" s="11">
+      <c r="K74">
         <v>29</v>
       </c>
       <c r="L74">
@@ -49073,7 +49076,7 @@
         <v>0.89</v>
       </c>
       <c r="F75">
-        <f>(I75+G75)/20</f>
+        <f t="shared" si="4"/>
         <v>0.45</v>
       </c>
       <c r="G75">
@@ -49083,13 +49086,13 @@
         <v>20</v>
       </c>
       <c r="I75">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>9</v>
       </c>
-      <c r="J75" s="11">
+      <c r="J75">
         <v>13</v>
       </c>
-      <c r="K75" s="11">
+      <c r="K75">
         <v>13</v>
       </c>
       <c r="L75">
@@ -49260,7 +49263,7 @@
         <v>0.91</v>
       </c>
       <c r="F76" s="6">
-        <f>(I76+G76)/20</f>
+        <f t="shared" si="4"/>
         <v>0.4</v>
       </c>
       <c r="G76" s="6">
@@ -49270,7 +49273,7 @@
         <v>20</v>
       </c>
       <c r="I76" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>6</v>
       </c>
       <c r="J76" s="6">
@@ -49447,7 +49450,7 @@
         <v>0.84</v>
       </c>
       <c r="F77">
-        <f>(I77+G77)/20</f>
+        <f t="shared" si="4"/>
         <v>0.9</v>
       </c>
       <c r="G77">
@@ -49457,13 +49460,13 @@
         <v>20</v>
       </c>
       <c r="I77">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>18</v>
       </c>
-      <c r="J77" s="11">
+      <c r="J77">
         <v>10</v>
       </c>
-      <c r="K77" s="11">
+      <c r="K77">
         <v>15</v>
       </c>
       <c r="L77">
@@ -49634,7 +49637,7 @@
         <v>0.92</v>
       </c>
       <c r="F78">
-        <f>(I78+G78)/20</f>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="G78">
@@ -49644,13 +49647,13 @@
         <v>20</v>
       </c>
       <c r="I78">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="J78" s="11">
+      <c r="J78">
         <v>8</v>
       </c>
-      <c r="K78" s="11">
+      <c r="K78">
         <v>13</v>
       </c>
       <c r="L78">
@@ -49821,7 +49824,7 @@
         <v>0.67</v>
       </c>
       <c r="F79">
-        <f>(I79+G79)/20</f>
+        <f t="shared" si="4"/>
         <v>0.35</v>
       </c>
       <c r="G79">
@@ -49831,13 +49834,13 @@
         <v>20</v>
       </c>
       <c r="I79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>7</v>
       </c>
-      <c r="J79" s="11">
+      <c r="J79">
         <v>13</v>
       </c>
-      <c r="K79" s="11">
+      <c r="K79">
         <v>13</v>
       </c>
       <c r="L79">
@@ -50008,7 +50011,7 @@
         <v>0.74</v>
       </c>
       <c r="F80">
-        <f>(I80+G80)/20</f>
+        <f t="shared" si="4"/>
         <v>0.75</v>
       </c>
       <c r="G80">
@@ -50018,13 +50021,13 @@
         <v>20</v>
       </c>
       <c r="I80">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>15</v>
       </c>
-      <c r="J80" s="11">
+      <c r="J80">
         <v>13</v>
       </c>
-      <c r="K80" s="11">
+      <c r="K80">
         <v>20</v>
       </c>
       <c r="L80">
@@ -50195,7 +50198,7 @@
         <v>0.87</v>
       </c>
       <c r="F81">
-        <f>(I81+G81)/20</f>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="G81">
@@ -50205,13 +50208,13 @@
         <v>20</v>
       </c>
       <c r="I81">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="J81" s="11">
+      <c r="J81">
         <v>13</v>
       </c>
-      <c r="K81" s="11">
+      <c r="K81">
         <v>24</v>
       </c>
       <c r="L81">
@@ -50382,7 +50385,7 @@
         <v>0.74</v>
       </c>
       <c r="F82">
-        <f>(I82+G82)/20</f>
+        <f t="shared" si="4"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="G82">
@@ -50392,13 +50395,13 @@
         <v>20</v>
       </c>
       <c r="I82">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>11</v>
       </c>
-      <c r="J82" s="11">
+      <c r="J82">
         <v>13</v>
       </c>
-      <c r="K82" s="11">
+      <c r="K82">
         <v>20</v>
       </c>
       <c r="L82">
@@ -50569,7 +50572,7 @@
         <v>0.93</v>
       </c>
       <c r="F83">
-        <f>(I83+G83)/20</f>
+        <f t="shared" si="4"/>
         <v>0.9</v>
       </c>
       <c r="G83">
@@ -50579,13 +50582,13 @@
         <v>20</v>
       </c>
       <c r="I83">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="J83" s="11">
+      <c r="J83">
         <v>13</v>
       </c>
-      <c r="K83" s="11">
+      <c r="K83">
         <v>2</v>
       </c>
       <c r="L83">
@@ -50756,7 +50759,7 @@
         <v>0.95</v>
       </c>
       <c r="F84">
-        <f>(I84+G84)/20</f>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="G84">
@@ -50766,13 +50769,13 @@
         <v>20</v>
       </c>
       <c r="I84">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="J84" s="11">
+      <c r="J84">
         <v>10</v>
       </c>
-      <c r="K84" s="11">
+      <c r="K84">
         <v>20</v>
       </c>
       <c r="L84">
@@ -50943,7 +50946,7 @@
         <v>0.93</v>
       </c>
       <c r="F85">
-        <f>(I85+G85)/20</f>
+        <f t="shared" si="4"/>
         <v>0.9</v>
       </c>
       <c r="G85">
@@ -50953,13 +50956,13 @@
         <v>20</v>
       </c>
       <c r="I85">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>18</v>
       </c>
-      <c r="J85" s="11">
+      <c r="J85">
         <v>13</v>
       </c>
-      <c r="K85" s="11">
+      <c r="K85">
         <v>20</v>
       </c>
       <c r="L85">
@@ -51130,7 +51133,7 @@
         <v>0.93</v>
       </c>
       <c r="F86">
-        <f>(I86+G86)/20</f>
+        <f t="shared" si="4"/>
         <v>0.95</v>
       </c>
       <c r="G86">
@@ -51140,13 +51143,13 @@
         <v>20</v>
       </c>
       <c r="I86">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>19</v>
       </c>
-      <c r="J86" s="11">
+      <c r="J86">
         <v>13</v>
       </c>
-      <c r="K86" s="11">
+      <c r="K86">
         <v>15</v>
       </c>
       <c r="L86">
@@ -51317,7 +51320,7 @@
         <v>0.93</v>
       </c>
       <c r="F87">
-        <f>(I87+G87)/20</f>
+        <f t="shared" si="4"/>
         <v>0.9</v>
       </c>
       <c r="G87">
@@ -51327,13 +51330,13 @@
         <v>20</v>
       </c>
       <c r="I87">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>18</v>
       </c>
-      <c r="J87" s="11">
+      <c r="J87">
         <v>13</v>
       </c>
-      <c r="K87" s="11">
+      <c r="K87">
         <v>20</v>
       </c>
       <c r="L87">
@@ -51504,7 +51507,7 @@
         <v>0.83</v>
       </c>
       <c r="F88">
-        <f>(I88+G88)/20</f>
+        <f t="shared" si="4"/>
         <v>0.75</v>
       </c>
       <c r="G88">
@@ -51514,13 +51517,13 @@
         <v>20</v>
       </c>
       <c r="I88">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>15</v>
       </c>
-      <c r="J88" s="11">
+      <c r="J88">
         <v>8</v>
       </c>
-      <c r="K88" s="11">
+      <c r="K88">
         <v>13</v>
       </c>
       <c r="L88">
@@ -51691,7 +51694,7 @@
         <v>0.52</v>
       </c>
       <c r="F89">
-        <f>(I89+G89)/20</f>
+        <f t="shared" si="4"/>
         <v>0.5</v>
       </c>
       <c r="G89">
@@ -51701,13 +51704,13 @@
         <v>20</v>
       </c>
       <c r="I89">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="J89" s="11">
+      <c r="J89">
         <v>10</v>
       </c>
-      <c r="K89" s="11">
+      <c r="K89">
         <v>22</v>
       </c>
       <c r="L89">
@@ -51878,7 +51881,7 @@
         <v>0.8</v>
       </c>
       <c r="F90">
-        <f>(I90+G90)/20</f>
+        <f t="shared" si="4"/>
         <v>0.85</v>
       </c>
       <c r="G90">
@@ -51888,13 +51891,13 @@
         <v>20</v>
       </c>
       <c r="I90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>17</v>
       </c>
-      <c r="J90" s="11">
+      <c r="J90">
         <v>10</v>
       </c>
-      <c r="K90" s="11">
+      <c r="K90">
         <v>20</v>
       </c>
       <c r="L90">
@@ -52065,7 +52068,7 @@
         <v>0.91</v>
       </c>
       <c r="F91">
-        <f>(I91+G91)/20</f>
+        <f t="shared" si="4"/>
         <v>0.3</v>
       </c>
       <c r="G91">
@@ -52075,13 +52078,13 @@
         <v>20</v>
       </c>
       <c r="I91">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>6</v>
       </c>
-      <c r="J91" s="11">
+      <c r="J91">
         <v>13</v>
       </c>
-      <c r="K91" s="11">
+      <c r="K91">
         <v>13</v>
       </c>
       <c r="L91">

</xml_diff>